<commit_message>
Add editted excel and sql querry
</commit_message>
<xml_diff>
--- a/Mina_Saeday/Saeday_Ex3A_tables.xlsx
+++ b/Mina_Saeday/Saeday_Ex3A_tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mina/DATA_Labs/W2_Workshop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mina/Desktop/yearup/W2_Workshop/Mina_Saeday/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81F8B517-468F-0C44-98B8-834854723AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5B9A9CF-15B5-764B-B34F-0068C1EB427D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="4" xr2:uid="{242FB6D9-B418-DF4D-8E59-86CAF174712F}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="4" xr2:uid="{242FB6D9-B418-DF4D-8E59-86CAF174712F}"/>
   </bookViews>
   <sheets>
     <sheet name="Customers" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
   <si>
     <t>customer_id</t>
   </si>
@@ -106,16 +106,66 @@
   </si>
   <si>
     <t>payment_method</t>
+  </si>
+  <si>
+    <t>Lana</t>
+  </si>
+  <si>
+    <t>Reed</t>
+  </si>
+  <si>
+    <t>555-123-5678</t>
+  </si>
+  <si>
+    <t>lana@gmail.com</t>
+  </si>
+  <si>
+    <t>123 jupyter st</t>
+  </si>
+  <si>
+    <t>Dom</t>
+  </si>
+  <si>
+    <t>Golder Retriever</t>
+  </si>
+  <si>
+    <t>Chris</t>
+  </si>
+  <si>
+    <t>Miller</t>
+  </si>
+  <si>
+    <t>676-222-889</t>
+  </si>
+  <si>
+    <t>chrismiler@gmal.com</t>
+  </si>
+  <si>
+    <t>9.00.00</t>
+  </si>
+  <si>
+    <t>morning walk in the park</t>
+  </si>
+  <si>
+    <t>Card</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -156,10 +206,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -167,8 +218,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -501,7 +558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E9FA459-1D79-0A4A-AAC7-9373E7ACAF7B}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -524,14 +581,37 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{C540A079-ADF5-314E-B1CA-CB57BBFBA4F9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1FA77F8-0BF0-0446-B0AD-809D7F5D221D}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -553,6 +633,29 @@
       <c r="F1" s="2" t="s">
         <v>0</v>
       </c>
+    </row>
+    <row r="2" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>65.5</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C3" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -561,7 +664,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DB7A862-6419-3A4B-AA96-9F8E5A0EA4E5}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -581,14 +684,34 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{EEDC9189-F1E6-B34E-AC98-A6FDC4214205}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D879B5B-EE73-9142-84AE-AE6DBC08F57E}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -612,6 +735,29 @@
       </c>
       <c r="G1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7">
+        <v>46128</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2">
+        <v>30</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -621,7 +767,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A773-F39C-B44B-940F-076A37152016}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -641,6 +787,23 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>25</v>
+      </c>
+      <c r="D2" s="7">
+        <v>46128</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>